<commit_message>
Add backtester, high-cap tokens, updated trade data
- backtest.ts: 8 strategies x 4 SL/TP configs, parameter sweep support
- data-collector: add BTC, ETH, SOL, XRP, SUI to WebSocket logging
- Updated xlsx with new PIPPIN + BLUAI trades (51 total)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bybit-exports/manual export from gui.xlsx
+++ b/bybit-exports/manual export from gui.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emile\dev\Venzen\venzen-finance\reverse-copy\bybit-exports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C10F3A3-5550-40CA-B24E-F2C9B3BBF7ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5152798C-99B4-4BEE-87DC-3085E9C05BAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2475" yWindow="3795" windowWidth="35325" windowHeight="15345" xr2:uid="{3AC7A350-C40F-4483-924C-032E8BEFD244}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="285">
   <si>
     <t xml:space="preserve">PIPPINUSDTLong </t>
   </si>
@@ -1375,6 +1375,123 @@
   <si>
     <r>
       <t>37dfce5c</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FFADB1B8"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t></t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">BLUAIUSDTShort </t>
+  </si>
+  <si>
+    <t>750 BLUAI</t>
+  </si>
+  <si>
+    <t>0.008201 USDT</t>
+  </si>
+  <si>
+    <t>0.008046 USDT</t>
+  </si>
+  <si>
+    <t>+0.1031 USDT‏(+16.36‎%)</t>
+  </si>
+  <si>
+    <t>0.01341577 USDT‏</t>
+  </si>
+  <si>
+    <r>
+      <t>4c14dea8</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FFADB1B8"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t></t>
+    </r>
+  </si>
+  <si>
+    <t>7,160 BLUAI</t>
+  </si>
+  <si>
+    <t>+0.9852 USDT‏(+16.40‎%)</t>
+  </si>
+  <si>
+    <t>0.12795349 USDT‏</t>
+  </si>
+  <si>
+    <r>
+      <t>2f1f16d4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FFADB1B8"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t></t>
+    </r>
+  </si>
+  <si>
+    <t>2,226 PIPPIN</t>
+  </si>
+  <si>
+    <t>0.05810 USDT</t>
+  </si>
+  <si>
+    <t>0.05618 USDT</t>
+  </si>
+  <si>
+    <t>+4.1340 USDT‏(+31.59‎%)</t>
+  </si>
+  <si>
+    <t>0.13991301 USDT‏</t>
+  </si>
+  <si>
+    <r>
+      <t>f339153b</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FFADB1B8"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t></t>
+    </r>
+  </si>
+  <si>
+    <t>1,170 PIPPIN</t>
+  </si>
+  <si>
+    <t>0.05970 USDT</t>
+  </si>
+  <si>
+    <t>0.05792 USDT</t>
+  </si>
+  <si>
+    <t>+2.0191 USDT‏(+28.57‎%)</t>
+  </si>
+  <si>
+    <t>0.06345447 USDT‏</t>
+  </si>
+  <si>
+    <r>
+      <t>36ba16df</t>
     </r>
     <r>
       <rPr>
@@ -1793,7 +1910,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBA3A39D-55F6-42CF-AA62-7C0E48D5CE99}">
-  <dimension ref="A1:J95"/>
+  <dimension ref="A1:J103"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.7109375" customWidth="1"/>
@@ -3999,62 +4116,570 @@
       <c r="I95" s="5"/>
       <c r="J95" s="7"/>
     </row>
+    <row r="96" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A96" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="B96" s="5" t="s">
+        <v>263</v>
+      </c>
+      <c r="C96" s="6">
+        <v>46107.639988425923</v>
+      </c>
+      <c r="D96" s="5" t="s">
+        <v>264</v>
+      </c>
+      <c r="E96" s="6">
+        <v>46107.647534722222</v>
+      </c>
+      <c r="F96" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="G96" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="H96" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="I96" s="5" t="s">
+        <v>267</v>
+      </c>
+      <c r="J96" s="7" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A97" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B97" s="5"/>
+      <c r="C97" s="6"/>
+      <c r="D97" s="5"/>
+      <c r="E97" s="6"/>
+      <c r="F97" s="5"/>
+      <c r="G97" s="5"/>
+      <c r="H97" s="5"/>
+      <c r="I97" s="5"/>
+      <c r="J97" s="7"/>
+    </row>
+    <row r="98" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A98" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="B98" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="C98" s="6">
+        <v>46107.639976851853</v>
+      </c>
+      <c r="D98" s="5" t="s">
+        <v>264</v>
+      </c>
+      <c r="E98" s="6">
+        <v>46107.647534722222</v>
+      </c>
+      <c r="F98" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="G98" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="H98" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="I98" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="J98" s="7" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A99" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B99" s="5"/>
+      <c r="C99" s="6"/>
+      <c r="D99" s="5"/>
+      <c r="E99" s="6"/>
+      <c r="F99" s="5"/>
+      <c r="G99" s="5"/>
+      <c r="H99" s="5"/>
+      <c r="I99" s="5"/>
+      <c r="J99" s="7"/>
+    </row>
+    <row r="100" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A100" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="B100" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="C100" s="6">
+        <v>46107.621851851851</v>
+      </c>
+      <c r="D100" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="E100" s="6">
+        <v>46107.631157407406</v>
+      </c>
+      <c r="F100" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="G100" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="H100" s="5" t="s">
+        <v>276</v>
+      </c>
+      <c r="I100" s="5" t="s">
+        <v>277</v>
+      </c>
+      <c r="J100" s="7" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A101" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B101" s="5"/>
+      <c r="C101" s="6"/>
+      <c r="D101" s="5"/>
+      <c r="E101" s="6"/>
+      <c r="F101" s="5"/>
+      <c r="G101" s="5"/>
+      <c r="H101" s="5"/>
+      <c r="I101" s="5"/>
+      <c r="J101" s="7"/>
+    </row>
+    <row r="102" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A102" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="B102" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="C102" s="6">
+        <v>46107.504166666666</v>
+      </c>
+      <c r="D102" s="5" t="s">
+        <v>280</v>
+      </c>
+      <c r="E102" s="6">
+        <v>46107.547349537039</v>
+      </c>
+      <c r="F102" s="5" t="s">
+        <v>281</v>
+      </c>
+      <c r="G102" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="H102" s="5" t="s">
+        <v>282</v>
+      </c>
+      <c r="I102" s="5" t="s">
+        <v>283</v>
+      </c>
+      <c r="J102" s="7" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A103" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B103" s="5"/>
+      <c r="C103" s="6"/>
+      <c r="D103" s="5"/>
+      <c r="E103" s="6"/>
+      <c r="F103" s="5"/>
+      <c r="G103" s="5"/>
+      <c r="H103" s="5"/>
+      <c r="I103" s="5"/>
+      <c r="J103" s="7"/>
+    </row>
   </sheetData>
-  <mergeCells count="414">
-    <mergeCell ref="B94:B95"/>
-    <mergeCell ref="C94:C95"/>
-    <mergeCell ref="D94:D95"/>
-    <mergeCell ref="E94:E95"/>
-    <mergeCell ref="F94:F95"/>
-    <mergeCell ref="G94:G95"/>
-    <mergeCell ref="H94:H95"/>
-    <mergeCell ref="I94:I95"/>
-    <mergeCell ref="J94:J95"/>
-    <mergeCell ref="B92:B93"/>
-    <mergeCell ref="C92:C93"/>
-    <mergeCell ref="D92:D93"/>
-    <mergeCell ref="E92:E93"/>
-    <mergeCell ref="F92:F93"/>
-    <mergeCell ref="G92:G93"/>
-    <mergeCell ref="H92:H93"/>
-    <mergeCell ref="I92:I93"/>
-    <mergeCell ref="J92:J93"/>
-    <mergeCell ref="B90:B91"/>
-    <mergeCell ref="C90:C91"/>
-    <mergeCell ref="D90:D91"/>
-    <mergeCell ref="E90:E91"/>
-    <mergeCell ref="F90:F91"/>
-    <mergeCell ref="G90:G91"/>
-    <mergeCell ref="H90:H91"/>
-    <mergeCell ref="I90:I91"/>
-    <mergeCell ref="J90:J91"/>
-    <mergeCell ref="H66:H67"/>
-    <mergeCell ref="I66:I67"/>
-    <mergeCell ref="J66:J67"/>
-    <mergeCell ref="B66:B67"/>
-    <mergeCell ref="C66:C67"/>
-    <mergeCell ref="D66:D67"/>
-    <mergeCell ref="E66:E67"/>
-    <mergeCell ref="F66:F67"/>
-    <mergeCell ref="G66:G67"/>
-    <mergeCell ref="B64:B65"/>
-    <mergeCell ref="C64:C65"/>
-    <mergeCell ref="D64:D65"/>
-    <mergeCell ref="E64:E65"/>
-    <mergeCell ref="F64:F65"/>
-    <mergeCell ref="G64:G65"/>
-    <mergeCell ref="H64:H65"/>
-    <mergeCell ref="I64:I65"/>
-    <mergeCell ref="J64:J65"/>
-    <mergeCell ref="B62:B63"/>
-    <mergeCell ref="C62:C63"/>
-    <mergeCell ref="D62:D63"/>
-    <mergeCell ref="E62:E63"/>
-    <mergeCell ref="F62:F63"/>
-    <mergeCell ref="G62:G63"/>
-    <mergeCell ref="H62:H63"/>
-    <mergeCell ref="I62:I63"/>
-    <mergeCell ref="J62:J63"/>
+  <mergeCells count="450">
+    <mergeCell ref="B102:B103"/>
+    <mergeCell ref="C102:C103"/>
+    <mergeCell ref="D102:D103"/>
+    <mergeCell ref="E102:E103"/>
+    <mergeCell ref="F102:F103"/>
+    <mergeCell ref="G102:G103"/>
+    <mergeCell ref="H102:H103"/>
+    <mergeCell ref="I102:I103"/>
+    <mergeCell ref="J102:J103"/>
+    <mergeCell ref="B100:B101"/>
+    <mergeCell ref="C100:C101"/>
+    <mergeCell ref="D100:D101"/>
+    <mergeCell ref="E100:E101"/>
+    <mergeCell ref="F100:F101"/>
+    <mergeCell ref="G100:G101"/>
+    <mergeCell ref="H100:H101"/>
+    <mergeCell ref="I100:I101"/>
+    <mergeCell ref="J100:J101"/>
+    <mergeCell ref="B98:B99"/>
+    <mergeCell ref="C98:C99"/>
+    <mergeCell ref="D98:D99"/>
+    <mergeCell ref="E98:E99"/>
+    <mergeCell ref="F98:F99"/>
+    <mergeCell ref="G98:G99"/>
+    <mergeCell ref="H98:H99"/>
+    <mergeCell ref="I98:I99"/>
+    <mergeCell ref="J98:J99"/>
+    <mergeCell ref="B96:B97"/>
+    <mergeCell ref="C96:C97"/>
+    <mergeCell ref="D96:D97"/>
+    <mergeCell ref="E96:E97"/>
+    <mergeCell ref="F96:F97"/>
+    <mergeCell ref="G96:G97"/>
+    <mergeCell ref="H96:H97"/>
+    <mergeCell ref="I96:I97"/>
+    <mergeCell ref="J96:J97"/>
+    <mergeCell ref="B88:B89"/>
+    <mergeCell ref="C88:C89"/>
+    <mergeCell ref="D88:D89"/>
+    <mergeCell ref="E88:E89"/>
+    <mergeCell ref="F88:F89"/>
+    <mergeCell ref="G88:G89"/>
+    <mergeCell ref="H88:H89"/>
+    <mergeCell ref="I88:I89"/>
+    <mergeCell ref="J88:J89"/>
+    <mergeCell ref="B86:B87"/>
+    <mergeCell ref="C86:C87"/>
+    <mergeCell ref="D86:D87"/>
+    <mergeCell ref="E86:E87"/>
+    <mergeCell ref="F86:F87"/>
+    <mergeCell ref="G86:G87"/>
+    <mergeCell ref="H86:H87"/>
+    <mergeCell ref="I86:I87"/>
+    <mergeCell ref="J86:J87"/>
+    <mergeCell ref="B84:B85"/>
+    <mergeCell ref="C84:C85"/>
+    <mergeCell ref="D84:D85"/>
+    <mergeCell ref="E84:E85"/>
+    <mergeCell ref="F84:F85"/>
+    <mergeCell ref="G84:G85"/>
+    <mergeCell ref="H84:H85"/>
+    <mergeCell ref="I84:I85"/>
+    <mergeCell ref="J84:J85"/>
+    <mergeCell ref="B82:B83"/>
+    <mergeCell ref="C82:C83"/>
+    <mergeCell ref="D82:D83"/>
+    <mergeCell ref="E82:E83"/>
+    <mergeCell ref="F82:F83"/>
+    <mergeCell ref="G82:G83"/>
+    <mergeCell ref="H82:H83"/>
+    <mergeCell ref="I82:I83"/>
+    <mergeCell ref="J82:J83"/>
+    <mergeCell ref="B80:B81"/>
+    <mergeCell ref="C80:C81"/>
+    <mergeCell ref="D80:D81"/>
+    <mergeCell ref="E80:E81"/>
+    <mergeCell ref="F80:F81"/>
+    <mergeCell ref="G80:G81"/>
+    <mergeCell ref="H80:H81"/>
+    <mergeCell ref="I80:I81"/>
+    <mergeCell ref="J80:J81"/>
+    <mergeCell ref="B78:B79"/>
+    <mergeCell ref="C78:C79"/>
+    <mergeCell ref="D78:D79"/>
+    <mergeCell ref="E78:E79"/>
+    <mergeCell ref="F78:F79"/>
+    <mergeCell ref="G78:G79"/>
+    <mergeCell ref="H78:H79"/>
+    <mergeCell ref="I78:I79"/>
+    <mergeCell ref="J78:J79"/>
+    <mergeCell ref="B76:B77"/>
+    <mergeCell ref="C76:C77"/>
+    <mergeCell ref="D76:D77"/>
+    <mergeCell ref="E76:E77"/>
+    <mergeCell ref="F76:F77"/>
+    <mergeCell ref="G76:G77"/>
+    <mergeCell ref="H76:H77"/>
+    <mergeCell ref="I76:I77"/>
+    <mergeCell ref="J76:J77"/>
+    <mergeCell ref="B74:B75"/>
+    <mergeCell ref="C74:C75"/>
+    <mergeCell ref="D74:D75"/>
+    <mergeCell ref="E74:E75"/>
+    <mergeCell ref="F74:F75"/>
+    <mergeCell ref="G74:G75"/>
+    <mergeCell ref="H74:H75"/>
+    <mergeCell ref="I74:I75"/>
+    <mergeCell ref="J74:J75"/>
+    <mergeCell ref="B72:B73"/>
+    <mergeCell ref="C72:C73"/>
+    <mergeCell ref="D72:D73"/>
+    <mergeCell ref="E72:E73"/>
+    <mergeCell ref="F72:F73"/>
+    <mergeCell ref="G72:G73"/>
+    <mergeCell ref="H72:H73"/>
+    <mergeCell ref="I72:I73"/>
+    <mergeCell ref="J72:J73"/>
+    <mergeCell ref="B70:B71"/>
+    <mergeCell ref="C70:C71"/>
+    <mergeCell ref="D70:D71"/>
+    <mergeCell ref="E70:E71"/>
+    <mergeCell ref="F70:F71"/>
+    <mergeCell ref="G70:G71"/>
+    <mergeCell ref="H70:H71"/>
+    <mergeCell ref="I70:I71"/>
+    <mergeCell ref="J70:J71"/>
+    <mergeCell ref="B68:B69"/>
+    <mergeCell ref="C68:C69"/>
+    <mergeCell ref="D68:D69"/>
+    <mergeCell ref="E68:E69"/>
+    <mergeCell ref="F68:F69"/>
+    <mergeCell ref="G68:G69"/>
+    <mergeCell ref="H68:H69"/>
+    <mergeCell ref="I68:I69"/>
+    <mergeCell ref="J68:J69"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="F4:F5"/>
+    <mergeCell ref="G4:G5"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="I4:I5"/>
+    <mergeCell ref="J4:J5"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="F6:F7"/>
+    <mergeCell ref="G6:G7"/>
+    <mergeCell ref="H6:H7"/>
+    <mergeCell ref="I6:I7"/>
+    <mergeCell ref="J6:J7"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="G8:G9"/>
+    <mergeCell ref="H8:H9"/>
+    <mergeCell ref="I8:I9"/>
+    <mergeCell ref="J8:J9"/>
+    <mergeCell ref="H10:H11"/>
+    <mergeCell ref="I10:I11"/>
+    <mergeCell ref="J10:J11"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="F12:F13"/>
+    <mergeCell ref="G12:G13"/>
+    <mergeCell ref="H12:H13"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="D10:D11"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="F10:F11"/>
+    <mergeCell ref="G10:G11"/>
+    <mergeCell ref="I12:I13"/>
+    <mergeCell ref="J12:J13"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="E14:E15"/>
+    <mergeCell ref="F14:F15"/>
+    <mergeCell ref="G14:G15"/>
+    <mergeCell ref="H14:H15"/>
+    <mergeCell ref="I14:I15"/>
+    <mergeCell ref="J14:J15"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="E16:E17"/>
+    <mergeCell ref="F16:F17"/>
+    <mergeCell ref="G16:G17"/>
+    <mergeCell ref="H16:H17"/>
+    <mergeCell ref="I16:I17"/>
+    <mergeCell ref="J16:J17"/>
+    <mergeCell ref="H18:H19"/>
+    <mergeCell ref="I18:I19"/>
+    <mergeCell ref="J18:J19"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="E20:E21"/>
+    <mergeCell ref="F20:F21"/>
+    <mergeCell ref="G20:G21"/>
+    <mergeCell ref="H20:H21"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="E18:E19"/>
+    <mergeCell ref="F18:F19"/>
+    <mergeCell ref="G18:G19"/>
+    <mergeCell ref="I20:I21"/>
+    <mergeCell ref="J20:J21"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="D22:D23"/>
+    <mergeCell ref="E22:E23"/>
+    <mergeCell ref="F22:F23"/>
+    <mergeCell ref="G22:G23"/>
+    <mergeCell ref="H22:H23"/>
+    <mergeCell ref="I22:I23"/>
+    <mergeCell ref="J22:J23"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="E24:E25"/>
+    <mergeCell ref="F24:F25"/>
+    <mergeCell ref="G24:G25"/>
+    <mergeCell ref="H24:H25"/>
+    <mergeCell ref="I24:I25"/>
+    <mergeCell ref="J24:J25"/>
+    <mergeCell ref="H26:H27"/>
+    <mergeCell ref="I26:I27"/>
+    <mergeCell ref="J26:J27"/>
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="C28:C29"/>
+    <mergeCell ref="D28:D29"/>
+    <mergeCell ref="E28:E29"/>
+    <mergeCell ref="F28:F29"/>
+    <mergeCell ref="G28:G29"/>
+    <mergeCell ref="H28:H29"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="C26:C27"/>
+    <mergeCell ref="D26:D27"/>
+    <mergeCell ref="E26:E27"/>
+    <mergeCell ref="F26:F27"/>
+    <mergeCell ref="G26:G27"/>
+    <mergeCell ref="I28:I29"/>
+    <mergeCell ref="J28:J29"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="C30:C31"/>
+    <mergeCell ref="D30:D31"/>
+    <mergeCell ref="E30:E31"/>
+    <mergeCell ref="F30:F31"/>
+    <mergeCell ref="G30:G31"/>
+    <mergeCell ref="H30:H31"/>
+    <mergeCell ref="I30:I31"/>
+    <mergeCell ref="J30:J31"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="C32:C33"/>
+    <mergeCell ref="D32:D33"/>
+    <mergeCell ref="E32:E33"/>
+    <mergeCell ref="F32:F33"/>
+    <mergeCell ref="G32:G33"/>
+    <mergeCell ref="H32:H33"/>
+    <mergeCell ref="I32:I33"/>
+    <mergeCell ref="J32:J33"/>
+    <mergeCell ref="H34:H35"/>
+    <mergeCell ref="I34:I35"/>
+    <mergeCell ref="J34:J35"/>
+    <mergeCell ref="B36:B37"/>
+    <mergeCell ref="C36:C37"/>
+    <mergeCell ref="D36:D37"/>
+    <mergeCell ref="E36:E37"/>
+    <mergeCell ref="F36:F37"/>
+    <mergeCell ref="G36:G37"/>
+    <mergeCell ref="H36:H37"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="C34:C35"/>
+    <mergeCell ref="D34:D35"/>
+    <mergeCell ref="E34:E35"/>
+    <mergeCell ref="F34:F35"/>
+    <mergeCell ref="G34:G35"/>
+    <mergeCell ref="I36:I37"/>
+    <mergeCell ref="J36:J37"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="D38:D39"/>
+    <mergeCell ref="E38:E39"/>
+    <mergeCell ref="F38:F39"/>
+    <mergeCell ref="G38:G39"/>
+    <mergeCell ref="H38:H39"/>
+    <mergeCell ref="I38:I39"/>
+    <mergeCell ref="J38:J39"/>
+    <mergeCell ref="B40:B41"/>
+    <mergeCell ref="C40:C41"/>
+    <mergeCell ref="D40:D41"/>
+    <mergeCell ref="E40:E41"/>
+    <mergeCell ref="F40:F41"/>
+    <mergeCell ref="G40:G41"/>
+    <mergeCell ref="H40:H41"/>
+    <mergeCell ref="I40:I41"/>
+    <mergeCell ref="J40:J41"/>
+    <mergeCell ref="H42:H43"/>
+    <mergeCell ref="I42:I43"/>
+    <mergeCell ref="J42:J43"/>
+    <mergeCell ref="B44:B45"/>
+    <mergeCell ref="C44:C45"/>
+    <mergeCell ref="D44:D45"/>
+    <mergeCell ref="E44:E45"/>
+    <mergeCell ref="F44:F45"/>
+    <mergeCell ref="G44:G45"/>
+    <mergeCell ref="H44:H45"/>
+    <mergeCell ref="B42:B43"/>
+    <mergeCell ref="C42:C43"/>
+    <mergeCell ref="D42:D43"/>
+    <mergeCell ref="E42:E43"/>
+    <mergeCell ref="F42:F43"/>
+    <mergeCell ref="G42:G43"/>
+    <mergeCell ref="I44:I45"/>
+    <mergeCell ref="J44:J45"/>
+    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="C46:C47"/>
+    <mergeCell ref="D46:D47"/>
+    <mergeCell ref="E46:E47"/>
+    <mergeCell ref="F46:F47"/>
+    <mergeCell ref="G46:G47"/>
+    <mergeCell ref="H46:H47"/>
+    <mergeCell ref="I46:I47"/>
+    <mergeCell ref="J46:J47"/>
+    <mergeCell ref="B48:B49"/>
+    <mergeCell ref="C48:C49"/>
+    <mergeCell ref="D48:D49"/>
+    <mergeCell ref="E48:E49"/>
+    <mergeCell ref="F48:F49"/>
+    <mergeCell ref="G48:G49"/>
+    <mergeCell ref="H48:H49"/>
+    <mergeCell ref="I48:I49"/>
+    <mergeCell ref="J48:J49"/>
+    <mergeCell ref="H50:H51"/>
+    <mergeCell ref="I50:I51"/>
+    <mergeCell ref="J50:J51"/>
+    <mergeCell ref="B52:B53"/>
+    <mergeCell ref="C52:C53"/>
+    <mergeCell ref="D52:D53"/>
+    <mergeCell ref="E52:E53"/>
+    <mergeCell ref="F52:F53"/>
+    <mergeCell ref="G52:G53"/>
+    <mergeCell ref="H52:H53"/>
+    <mergeCell ref="B50:B51"/>
+    <mergeCell ref="C50:C51"/>
+    <mergeCell ref="D50:D51"/>
+    <mergeCell ref="E50:E51"/>
+    <mergeCell ref="F50:F51"/>
+    <mergeCell ref="G50:G51"/>
+    <mergeCell ref="I52:I53"/>
+    <mergeCell ref="J52:J53"/>
+    <mergeCell ref="B54:B55"/>
+    <mergeCell ref="C54:C55"/>
+    <mergeCell ref="D54:D55"/>
+    <mergeCell ref="E54:E55"/>
+    <mergeCell ref="F54:F55"/>
+    <mergeCell ref="G54:G55"/>
+    <mergeCell ref="H54:H55"/>
+    <mergeCell ref="I54:I55"/>
+    <mergeCell ref="J54:J55"/>
+    <mergeCell ref="B56:B57"/>
+    <mergeCell ref="C56:C57"/>
+    <mergeCell ref="D56:D57"/>
+    <mergeCell ref="E56:E57"/>
+    <mergeCell ref="F56:F57"/>
+    <mergeCell ref="G56:G57"/>
+    <mergeCell ref="H56:H57"/>
+    <mergeCell ref="I56:I57"/>
+    <mergeCell ref="J56:J57"/>
     <mergeCell ref="H58:H59"/>
     <mergeCell ref="I58:I59"/>
     <mergeCell ref="J58:J59"/>
@@ -4073,348 +4698,60 @@
     <mergeCell ref="G58:G59"/>
     <mergeCell ref="I60:I61"/>
     <mergeCell ref="J60:J61"/>
-    <mergeCell ref="B56:B57"/>
-    <mergeCell ref="C56:C57"/>
-    <mergeCell ref="D56:D57"/>
-    <mergeCell ref="E56:E57"/>
-    <mergeCell ref="F56:F57"/>
-    <mergeCell ref="G56:G57"/>
-    <mergeCell ref="H56:H57"/>
-    <mergeCell ref="I56:I57"/>
-    <mergeCell ref="J56:J57"/>
-    <mergeCell ref="B54:B55"/>
-    <mergeCell ref="C54:C55"/>
-    <mergeCell ref="D54:D55"/>
-    <mergeCell ref="E54:E55"/>
-    <mergeCell ref="F54:F55"/>
-    <mergeCell ref="G54:G55"/>
-    <mergeCell ref="H54:H55"/>
-    <mergeCell ref="I54:I55"/>
-    <mergeCell ref="J54:J55"/>
-    <mergeCell ref="H50:H51"/>
-    <mergeCell ref="I50:I51"/>
-    <mergeCell ref="J50:J51"/>
-    <mergeCell ref="B52:B53"/>
-    <mergeCell ref="C52:C53"/>
-    <mergeCell ref="D52:D53"/>
-    <mergeCell ref="E52:E53"/>
-    <mergeCell ref="F52:F53"/>
-    <mergeCell ref="G52:G53"/>
-    <mergeCell ref="H52:H53"/>
-    <mergeCell ref="B50:B51"/>
-    <mergeCell ref="C50:C51"/>
-    <mergeCell ref="D50:D51"/>
-    <mergeCell ref="E50:E51"/>
-    <mergeCell ref="F50:F51"/>
-    <mergeCell ref="G50:G51"/>
-    <mergeCell ref="I52:I53"/>
-    <mergeCell ref="J52:J53"/>
-    <mergeCell ref="B48:B49"/>
-    <mergeCell ref="C48:C49"/>
-    <mergeCell ref="D48:D49"/>
-    <mergeCell ref="E48:E49"/>
-    <mergeCell ref="F48:F49"/>
-    <mergeCell ref="G48:G49"/>
-    <mergeCell ref="H48:H49"/>
-    <mergeCell ref="I48:I49"/>
-    <mergeCell ref="J48:J49"/>
-    <mergeCell ref="B46:B47"/>
-    <mergeCell ref="C46:C47"/>
-    <mergeCell ref="D46:D47"/>
-    <mergeCell ref="E46:E47"/>
-    <mergeCell ref="F46:F47"/>
-    <mergeCell ref="G46:G47"/>
-    <mergeCell ref="H46:H47"/>
-    <mergeCell ref="I46:I47"/>
-    <mergeCell ref="J46:J47"/>
-    <mergeCell ref="H42:H43"/>
-    <mergeCell ref="I42:I43"/>
-    <mergeCell ref="J42:J43"/>
-    <mergeCell ref="B44:B45"/>
-    <mergeCell ref="C44:C45"/>
-    <mergeCell ref="D44:D45"/>
-    <mergeCell ref="E44:E45"/>
-    <mergeCell ref="F44:F45"/>
-    <mergeCell ref="G44:G45"/>
-    <mergeCell ref="H44:H45"/>
-    <mergeCell ref="B42:B43"/>
-    <mergeCell ref="C42:C43"/>
-    <mergeCell ref="D42:D43"/>
-    <mergeCell ref="E42:E43"/>
-    <mergeCell ref="F42:F43"/>
-    <mergeCell ref="G42:G43"/>
-    <mergeCell ref="I44:I45"/>
-    <mergeCell ref="J44:J45"/>
-    <mergeCell ref="B40:B41"/>
-    <mergeCell ref="C40:C41"/>
-    <mergeCell ref="D40:D41"/>
-    <mergeCell ref="E40:E41"/>
-    <mergeCell ref="F40:F41"/>
-    <mergeCell ref="G40:G41"/>
-    <mergeCell ref="H40:H41"/>
-    <mergeCell ref="I40:I41"/>
-    <mergeCell ref="J40:J41"/>
-    <mergeCell ref="B38:B39"/>
-    <mergeCell ref="C38:C39"/>
-    <mergeCell ref="D38:D39"/>
-    <mergeCell ref="E38:E39"/>
-    <mergeCell ref="F38:F39"/>
-    <mergeCell ref="G38:G39"/>
-    <mergeCell ref="H38:H39"/>
-    <mergeCell ref="I38:I39"/>
-    <mergeCell ref="J38:J39"/>
-    <mergeCell ref="H34:H35"/>
-    <mergeCell ref="I34:I35"/>
-    <mergeCell ref="J34:J35"/>
-    <mergeCell ref="B36:B37"/>
-    <mergeCell ref="C36:C37"/>
-    <mergeCell ref="D36:D37"/>
-    <mergeCell ref="E36:E37"/>
-    <mergeCell ref="F36:F37"/>
-    <mergeCell ref="G36:G37"/>
-    <mergeCell ref="H36:H37"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="C34:C35"/>
-    <mergeCell ref="D34:D35"/>
-    <mergeCell ref="E34:E35"/>
-    <mergeCell ref="F34:F35"/>
-    <mergeCell ref="G34:G35"/>
-    <mergeCell ref="I36:I37"/>
-    <mergeCell ref="J36:J37"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="C32:C33"/>
-    <mergeCell ref="D32:D33"/>
-    <mergeCell ref="E32:E33"/>
-    <mergeCell ref="F32:F33"/>
-    <mergeCell ref="G32:G33"/>
-    <mergeCell ref="H32:H33"/>
-    <mergeCell ref="I32:I33"/>
-    <mergeCell ref="J32:J33"/>
-    <mergeCell ref="B30:B31"/>
-    <mergeCell ref="C30:C31"/>
-    <mergeCell ref="D30:D31"/>
-    <mergeCell ref="E30:E31"/>
-    <mergeCell ref="F30:F31"/>
-    <mergeCell ref="G30:G31"/>
-    <mergeCell ref="H30:H31"/>
-    <mergeCell ref="I30:I31"/>
-    <mergeCell ref="J30:J31"/>
-    <mergeCell ref="H26:H27"/>
-    <mergeCell ref="I26:I27"/>
-    <mergeCell ref="J26:J27"/>
-    <mergeCell ref="B28:B29"/>
-    <mergeCell ref="C28:C29"/>
-    <mergeCell ref="D28:D29"/>
-    <mergeCell ref="E28:E29"/>
-    <mergeCell ref="F28:F29"/>
-    <mergeCell ref="G28:G29"/>
-    <mergeCell ref="H28:H29"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="C26:C27"/>
-    <mergeCell ref="D26:D27"/>
-    <mergeCell ref="E26:E27"/>
-    <mergeCell ref="F26:F27"/>
-    <mergeCell ref="G26:G27"/>
-    <mergeCell ref="I28:I29"/>
-    <mergeCell ref="J28:J29"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="E24:E25"/>
-    <mergeCell ref="F24:F25"/>
-    <mergeCell ref="G24:G25"/>
-    <mergeCell ref="H24:H25"/>
-    <mergeCell ref="I24:I25"/>
-    <mergeCell ref="J24:J25"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="D22:D23"/>
-    <mergeCell ref="E22:E23"/>
-    <mergeCell ref="F22:F23"/>
-    <mergeCell ref="G22:G23"/>
-    <mergeCell ref="H22:H23"/>
-    <mergeCell ref="I22:I23"/>
-    <mergeCell ref="J22:J23"/>
-    <mergeCell ref="H18:H19"/>
-    <mergeCell ref="I18:I19"/>
-    <mergeCell ref="J18:J19"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="E20:E21"/>
-    <mergeCell ref="F20:F21"/>
-    <mergeCell ref="G20:G21"/>
-    <mergeCell ref="H20:H21"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="D18:D19"/>
-    <mergeCell ref="E18:E19"/>
-    <mergeCell ref="F18:F19"/>
-    <mergeCell ref="G18:G19"/>
-    <mergeCell ref="I20:I21"/>
-    <mergeCell ref="J20:J21"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="E16:E17"/>
-    <mergeCell ref="F16:F17"/>
-    <mergeCell ref="G16:G17"/>
-    <mergeCell ref="H16:H17"/>
-    <mergeCell ref="I16:I17"/>
-    <mergeCell ref="J16:J17"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="E14:E15"/>
-    <mergeCell ref="F14:F15"/>
-    <mergeCell ref="G14:G15"/>
-    <mergeCell ref="H14:H15"/>
-    <mergeCell ref="I14:I15"/>
-    <mergeCell ref="J14:J15"/>
-    <mergeCell ref="H10:H11"/>
-    <mergeCell ref="I10:I11"/>
-    <mergeCell ref="J10:J11"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="D12:D13"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="F12:F13"/>
-    <mergeCell ref="G12:G13"/>
-    <mergeCell ref="H12:H13"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="D10:D11"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="F10:F11"/>
-    <mergeCell ref="G10:G11"/>
-    <mergeCell ref="I12:I13"/>
-    <mergeCell ref="J12:J13"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="E8:E9"/>
-    <mergeCell ref="F8:F9"/>
-    <mergeCell ref="G8:G9"/>
-    <mergeCell ref="H8:H9"/>
-    <mergeCell ref="I8:I9"/>
-    <mergeCell ref="J8:J9"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="E6:E7"/>
-    <mergeCell ref="F6:F7"/>
-    <mergeCell ref="G6:G7"/>
-    <mergeCell ref="H6:H7"/>
-    <mergeCell ref="I6:I7"/>
-    <mergeCell ref="J6:J7"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="F4:F5"/>
-    <mergeCell ref="G4:G5"/>
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="I4:I5"/>
-    <mergeCell ref="J4:J5"/>
-    <mergeCell ref="B68:B69"/>
-    <mergeCell ref="C68:C69"/>
-    <mergeCell ref="D68:D69"/>
-    <mergeCell ref="E68:E69"/>
-    <mergeCell ref="F68:F69"/>
-    <mergeCell ref="G68:G69"/>
-    <mergeCell ref="H68:H69"/>
-    <mergeCell ref="I68:I69"/>
-    <mergeCell ref="J68:J69"/>
-    <mergeCell ref="B70:B71"/>
-    <mergeCell ref="C70:C71"/>
-    <mergeCell ref="D70:D71"/>
-    <mergeCell ref="E70:E71"/>
-    <mergeCell ref="F70:F71"/>
-    <mergeCell ref="G70:G71"/>
-    <mergeCell ref="H70:H71"/>
-    <mergeCell ref="I70:I71"/>
-    <mergeCell ref="J70:J71"/>
-    <mergeCell ref="B72:B73"/>
-    <mergeCell ref="C72:C73"/>
-    <mergeCell ref="D72:D73"/>
-    <mergeCell ref="E72:E73"/>
-    <mergeCell ref="F72:F73"/>
-    <mergeCell ref="G72:G73"/>
-    <mergeCell ref="H72:H73"/>
-    <mergeCell ref="I72:I73"/>
-    <mergeCell ref="J72:J73"/>
-    <mergeCell ref="B74:B75"/>
-    <mergeCell ref="C74:C75"/>
-    <mergeCell ref="D74:D75"/>
-    <mergeCell ref="E74:E75"/>
-    <mergeCell ref="F74:F75"/>
-    <mergeCell ref="G74:G75"/>
-    <mergeCell ref="H74:H75"/>
-    <mergeCell ref="I74:I75"/>
-    <mergeCell ref="J74:J75"/>
-    <mergeCell ref="B76:B77"/>
-    <mergeCell ref="C76:C77"/>
-    <mergeCell ref="D76:D77"/>
-    <mergeCell ref="E76:E77"/>
-    <mergeCell ref="F76:F77"/>
-    <mergeCell ref="G76:G77"/>
-    <mergeCell ref="H76:H77"/>
-    <mergeCell ref="I76:I77"/>
-    <mergeCell ref="J76:J77"/>
-    <mergeCell ref="B78:B79"/>
-    <mergeCell ref="C78:C79"/>
-    <mergeCell ref="D78:D79"/>
-    <mergeCell ref="E78:E79"/>
-    <mergeCell ref="F78:F79"/>
-    <mergeCell ref="G78:G79"/>
-    <mergeCell ref="H78:H79"/>
-    <mergeCell ref="I78:I79"/>
-    <mergeCell ref="J78:J79"/>
-    <mergeCell ref="B80:B81"/>
-    <mergeCell ref="C80:C81"/>
-    <mergeCell ref="D80:D81"/>
-    <mergeCell ref="E80:E81"/>
-    <mergeCell ref="F80:F81"/>
-    <mergeCell ref="G80:G81"/>
-    <mergeCell ref="H80:H81"/>
-    <mergeCell ref="I80:I81"/>
-    <mergeCell ref="J80:J81"/>
-    <mergeCell ref="B82:B83"/>
-    <mergeCell ref="C82:C83"/>
-    <mergeCell ref="D82:D83"/>
-    <mergeCell ref="E82:E83"/>
-    <mergeCell ref="F82:F83"/>
-    <mergeCell ref="G82:G83"/>
-    <mergeCell ref="H82:H83"/>
-    <mergeCell ref="I82:I83"/>
-    <mergeCell ref="J82:J83"/>
-    <mergeCell ref="B84:B85"/>
-    <mergeCell ref="C84:C85"/>
-    <mergeCell ref="D84:D85"/>
-    <mergeCell ref="E84:E85"/>
-    <mergeCell ref="F84:F85"/>
-    <mergeCell ref="G84:G85"/>
-    <mergeCell ref="H84:H85"/>
-    <mergeCell ref="I84:I85"/>
-    <mergeCell ref="J84:J85"/>
-    <mergeCell ref="B86:B87"/>
-    <mergeCell ref="C86:C87"/>
-    <mergeCell ref="D86:D87"/>
-    <mergeCell ref="E86:E87"/>
-    <mergeCell ref="F86:F87"/>
-    <mergeCell ref="G86:G87"/>
-    <mergeCell ref="H86:H87"/>
-    <mergeCell ref="I86:I87"/>
-    <mergeCell ref="J86:J87"/>
-    <mergeCell ref="B88:B89"/>
-    <mergeCell ref="C88:C89"/>
-    <mergeCell ref="D88:D89"/>
-    <mergeCell ref="E88:E89"/>
-    <mergeCell ref="F88:F89"/>
-    <mergeCell ref="G88:G89"/>
-    <mergeCell ref="H88:H89"/>
-    <mergeCell ref="I88:I89"/>
-    <mergeCell ref="J88:J89"/>
+    <mergeCell ref="B62:B63"/>
+    <mergeCell ref="C62:C63"/>
+    <mergeCell ref="D62:D63"/>
+    <mergeCell ref="E62:E63"/>
+    <mergeCell ref="F62:F63"/>
+    <mergeCell ref="G62:G63"/>
+    <mergeCell ref="H62:H63"/>
+    <mergeCell ref="I62:I63"/>
+    <mergeCell ref="J62:J63"/>
+    <mergeCell ref="B64:B65"/>
+    <mergeCell ref="C64:C65"/>
+    <mergeCell ref="D64:D65"/>
+    <mergeCell ref="E64:E65"/>
+    <mergeCell ref="F64:F65"/>
+    <mergeCell ref="G64:G65"/>
+    <mergeCell ref="H64:H65"/>
+    <mergeCell ref="I64:I65"/>
+    <mergeCell ref="J64:J65"/>
+    <mergeCell ref="H66:H67"/>
+    <mergeCell ref="I66:I67"/>
+    <mergeCell ref="J66:J67"/>
+    <mergeCell ref="B66:B67"/>
+    <mergeCell ref="C66:C67"/>
+    <mergeCell ref="D66:D67"/>
+    <mergeCell ref="E66:E67"/>
+    <mergeCell ref="F66:F67"/>
+    <mergeCell ref="G66:G67"/>
+    <mergeCell ref="B90:B91"/>
+    <mergeCell ref="C90:C91"/>
+    <mergeCell ref="D90:D91"/>
+    <mergeCell ref="E90:E91"/>
+    <mergeCell ref="F90:F91"/>
+    <mergeCell ref="G90:G91"/>
+    <mergeCell ref="H90:H91"/>
+    <mergeCell ref="I90:I91"/>
+    <mergeCell ref="J90:J91"/>
+    <mergeCell ref="B92:B93"/>
+    <mergeCell ref="C92:C93"/>
+    <mergeCell ref="D92:D93"/>
+    <mergeCell ref="E92:E93"/>
+    <mergeCell ref="F92:F93"/>
+    <mergeCell ref="G92:G93"/>
+    <mergeCell ref="H92:H93"/>
+    <mergeCell ref="I92:I93"/>
+    <mergeCell ref="J92:J93"/>
+    <mergeCell ref="B94:B95"/>
+    <mergeCell ref="C94:C95"/>
+    <mergeCell ref="D94:D95"/>
+    <mergeCell ref="E94:E95"/>
+    <mergeCell ref="F94:F95"/>
+    <mergeCell ref="G94:G95"/>
+    <mergeCell ref="H94:H95"/>
+    <mergeCell ref="I94:I95"/>
+    <mergeCell ref="J94:J95"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>

</xml_diff>